<commit_message>
backup - includes Leiden clustering, new output images and code for FCM system modelling (ensemble simulation and stable state analysis)
</commit_message>
<xml_diff>
--- a/Interviews/Interviews.xlsx
+++ b/Interviews/Interviews.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoe-my.sharepoint.com/personal/s1512187_ed_ac_uk/Documents/Documents/PhD/Interviews/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoe-my.sharepoint.com/personal/s1512187_ed_ac_uk/Documents/Documents/PhD/FCMs/interviews/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{83584A76-9DDA-428C-A035-998435B570EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38EE92FF-A2D5-4F27-AE5C-BE9699B1EAC2}"/>
+  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{83584A76-9DDA-428C-A035-998435B570EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{937705A0-A998-4CDB-8827-7D8ABCDE1E17}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interviews" sheetId="1" r:id="rId1"/>
     <sheet name="Transcriptions" sheetId="2" r:id="rId2"/>
+    <sheet name="Interviews_tidy" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="199">
   <si>
     <t>Date</t>
   </si>
@@ -458,6 +462,180 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>10_transcript</t>
+  </si>
+  <si>
+    <t>11_transcript</t>
+  </si>
+  <si>
+    <t>12_transcript</t>
+  </si>
+  <si>
+    <t>14_transcript</t>
+  </si>
+  <si>
+    <t>15_transcript</t>
+  </si>
+  <si>
+    <t>16_transcript</t>
+  </si>
+  <si>
+    <t>17_transcript</t>
+  </si>
+  <si>
+    <t>18_transcript</t>
+  </si>
+  <si>
+    <t>19_transcript</t>
+  </si>
+  <si>
+    <t>20_transcript</t>
+  </si>
+  <si>
+    <t>21_transcript</t>
+  </si>
+  <si>
+    <t>22_transcript</t>
+  </si>
+  <si>
+    <t>23_transcript</t>
+  </si>
+  <si>
+    <t>24_transcript</t>
+  </si>
+  <si>
+    <t>25_transcript</t>
+  </si>
+  <si>
+    <t>26_transcript</t>
+  </si>
+  <si>
+    <t>27_transcript</t>
+  </si>
+  <si>
+    <t>28_transcript</t>
+  </si>
+  <si>
+    <t>29_transcript</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>transcribed</t>
+  </si>
+  <si>
+    <t>05_transcript</t>
+  </si>
+  <si>
+    <t>06_transcript</t>
+  </si>
+  <si>
+    <t>13_part1_transcript</t>
+  </si>
+  <si>
+    <t>13_part2_transcript</t>
+  </si>
+  <si>
+    <t>35_transcript</t>
+  </si>
+  <si>
+    <t>36_transcript</t>
+  </si>
+  <si>
+    <t>30_transcript</t>
+  </si>
+  <si>
+    <t>31_transcript</t>
+  </si>
+  <si>
+    <t>32_transcript</t>
+  </si>
+  <si>
+    <t>33_transcript</t>
+  </si>
+  <si>
+    <t>34_transcript</t>
+  </si>
+  <si>
+    <t>Martin</t>
+  </si>
+  <si>
+    <t>Length (mins)</t>
+  </si>
+  <si>
+    <t>tranche</t>
+  </si>
+  <si>
+    <t>Jennifer</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Stakeholder</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>Secondary</t>
+  </si>
+  <si>
+    <t>Community Elder</t>
+  </si>
+  <si>
+    <t>Abba Errega (Water Manager)</t>
+  </si>
+  <si>
+    <t>Pastoralism expert with focus on markets</t>
+  </si>
+  <si>
+    <t>Senior Animal Health Officer</t>
+  </si>
+  <si>
+    <t>CEO of NGO working on pastoralism</t>
+  </si>
+  <si>
+    <t>Veterinarian and government employee</t>
+  </si>
+  <si>
+    <t>Community Elder &amp; herder</t>
+  </si>
+  <si>
+    <t>Health Professional working in government dispensary</t>
+  </si>
+  <si>
+    <t>Management Committee member of a Women's Group</t>
+  </si>
+  <si>
+    <t>Secretary of a Women's Group</t>
+  </si>
+  <si>
+    <t>Chief</t>
+  </si>
+  <si>
+    <t>Widow</t>
+  </si>
+  <si>
+    <t>CEO of Sub County Referral Hospital</t>
+  </si>
+  <si>
+    <t>Deputy Director of NGO working in Marsabit</t>
+  </si>
+  <si>
+    <t>Employee in County Government Dept. Water, Environment and Natural Resources</t>
+  </si>
+  <si>
+    <t>Employee in County Government Dept. Public Health</t>
+  </si>
+  <si>
+    <t>Man</t>
+  </si>
+  <si>
+    <t>Woman</t>
   </si>
 </sst>
 </file>
@@ -493,10 +671,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2028,13 +2208,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A07F7810-3D79-4E76-92EF-6D62A59CE228}">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7265625" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2059,8 +2241,50 @@
       <c r="H1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>160</v>
+      </c>
+      <c r="J1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K1" t="s">
+        <v>173</v>
+      </c>
+      <c r="L1" t="s">
+        <v>174</v>
+      </c>
+      <c r="M1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O1" t="s">
+        <v>133</v>
+      </c>
+      <c r="P1" t="s">
+        <v>134</v>
+      </c>
+      <c r="R1" t="s">
+        <v>176</v>
+      </c>
+      <c r="S1" t="s">
+        <v>174</v>
+      </c>
+      <c r="T1" t="s">
+        <v>69</v>
+      </c>
+      <c r="U1" t="s">
+        <v>73</v>
+      </c>
+      <c r="V1" t="s">
+        <v>133</v>
+      </c>
+      <c r="W1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2085,8 +2309,23 @@
         <f>F2-SUM(G$2:G2)</f>
         <v>2820</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" t="s">
+        <v>161</v>
+      </c>
+      <c r="N2">
+        <f>SUM(M$2:M2)</f>
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <f>S2*35</f>
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <f>SUM(T$2:T2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2100,7 +2339,7 @@
         <v>44</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E17" si="0">D3*30</f>
+        <f t="shared" ref="E3:E39" si="0">D3*30</f>
         <v>1320</v>
       </c>
       <c r="F3">
@@ -2111,8 +2350,23 @@
         <f>F3-SUM(G$2:G3)</f>
         <v>4140</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3" t="s">
+        <v>161</v>
+      </c>
+      <c r="N3">
+        <f>SUM(M$2:M3)</f>
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <f t="shared" ref="T3:T39" si="1">S3*35</f>
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <f>SUM(T$2:T3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2140,8 +2394,23 @@
         <f>F4-SUM(G$2:G4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4" t="s">
+        <v>161</v>
+      </c>
+      <c r="N4">
+        <f>SUM(M$2:M4)</f>
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <f>SUM(T$2:T4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2166,8 +2435,24 @@
         <f>F5-SUM(G$2:G5)</f>
         <v>2580</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5" t="s">
+        <v>161</v>
+      </c>
+      <c r="K5" s="3"/>
+      <c r="N5">
+        <f>SUM(M$2:M5)</f>
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <f>SUM(T$2:T5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2192,10 +2477,32 @@
         <f>F6-SUM(G$2:G6)</f>
         <v>5280</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I6" t="s">
+        <v>161</v>
+      </c>
+      <c r="K6" s="3"/>
+      <c r="N6">
+        <f>SUM(M$2:M6)</f>
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <f>SUM(T$2:T6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C7" s="2">
+        <v>5.6944444444444443E-2</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
@@ -2209,10 +2516,42 @@
         <f>F7-SUM(G$2:G7)</f>
         <v>5280</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="K7" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L7">
+        <v>82</v>
+      </c>
+      <c r="M7">
+        <f>L7*30</f>
+        <v>2460</v>
+      </c>
+      <c r="N7">
+        <f>SUM(M$2:M7)</f>
+        <v>2460</v>
+      </c>
+      <c r="O7" s="1">
+        <v>45925</v>
+      </c>
+      <c r="R7" s="3"/>
+      <c r="T7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <f>SUM(T$2:T7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" s="2">
+        <v>4.6527777777777779E-2</v>
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
@@ -2226,8 +2565,34 @@
         <f>F8-SUM(G$2:G8)</f>
         <v>5280</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="K8" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L8">
+        <v>67</v>
+      </c>
+      <c r="M8">
+        <f t="shared" ref="M8:M34" si="2">L8*30</f>
+        <v>2010</v>
+      </c>
+      <c r="N8">
+        <f>SUM(M$2:M8)</f>
+        <v>4470</v>
+      </c>
+      <c r="O8" s="1">
+        <v>45936</v>
+      </c>
+      <c r="R8" s="3"/>
+      <c r="T8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <f>SUM(T$2:T8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2252,8 +2617,28 @@
         <f>F9-SUM(G$2:G9)</f>
         <v>7770</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9" t="s">
+        <v>161</v>
+      </c>
+      <c r="K9" s="3"/>
+      <c r="M9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <f>SUM(M$2:M9)</f>
+        <v>4470</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <f>SUM(T$2:T9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2278,8 +2663,28 @@
         <f>F10-SUM(G$2:G10)</f>
         <v>10080</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I10" t="s">
+        <v>161</v>
+      </c>
+      <c r="K10" s="3"/>
+      <c r="M10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <f>SUM(M$2:M10)</f>
+        <v>4470</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <f>SUM(T$2:T10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2307,78 +2712,225 @@
         <f>F11-SUM(G$2:G11)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11" t="s">
+        <v>161</v>
+      </c>
+      <c r="K11" s="3"/>
+      <c r="M11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <f>SUM(M$2:M11)</f>
+        <v>4470</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <f>SUM(T$2:T11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>10</v>
       </c>
+      <c r="B12" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="2">
+        <v>5.347222222222222E-2</v>
+      </c>
+      <c r="D12">
+        <v>77</v>
+      </c>
       <c r="E12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2310</v>
       </c>
       <c r="F12">
         <f>SUM(E$2:E12)</f>
-        <v>19500</v>
+        <v>21810</v>
       </c>
       <c r="H12">
         <f>F12-SUM(G$2:G12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>2310</v>
+      </c>
+      <c r="I12" t="s">
+        <v>161</v>
+      </c>
+      <c r="K12" s="3"/>
+      <c r="M12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <f>SUM(M$2:M12)</f>
+        <v>4470</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <f>SUM(T$2:T12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>11</v>
       </c>
+      <c r="B13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2.7777777777777776E-2</v>
+      </c>
+      <c r="D13">
+        <v>40</v>
+      </c>
       <c r="E13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F13">
         <f>SUM(E$2:E13)</f>
-        <v>19500</v>
+        <v>23010</v>
       </c>
       <c r="H13">
         <f>F13-SUM(G$2:G13)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3510</v>
+      </c>
+      <c r="I13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K13" s="3"/>
+      <c r="M13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <f>SUM(M$2:M13)</f>
+        <v>4470</v>
+      </c>
+      <c r="R13" s="3"/>
+      <c r="T13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <f>SUM(T$2:T13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>12</v>
       </c>
+      <c r="B14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" s="2">
+        <v>4.8611111111111112E-2</v>
+      </c>
+      <c r="D14">
+        <v>70</v>
+      </c>
       <c r="E14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2100</v>
       </c>
       <c r="F14">
         <f>SUM(E$2:E14)</f>
-        <v>19500</v>
+        <v>25110</v>
       </c>
       <c r="H14">
         <f>F14-SUM(G$2:G14)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+        <v>5610</v>
+      </c>
+      <c r="I14" t="s">
+        <v>161</v>
+      </c>
+      <c r="K14" s="3"/>
+      <c r="M14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <f>SUM(M$2:M14)</f>
+        <v>4470</v>
+      </c>
+      <c r="R14" s="3"/>
+      <c r="T14">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <f>SUM(T$2:T14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>13</v>
       </c>
+      <c r="B15" t="s">
+        <v>164</v>
+      </c>
+      <c r="C15" s="2">
+        <v>4.2361111111111113E-2</v>
+      </c>
       <c r="E15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F15">
         <f>SUM(E$2:E15)</f>
-        <v>19500</v>
+        <v>25110</v>
       </c>
       <c r="H15">
         <f>F15-SUM(G$2:G15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+        <v>5610</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L15">
+        <v>61</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="2"/>
+        <v>1830</v>
+      </c>
+      <c r="N15">
+        <f>SUM(M$2:M15)</f>
+        <v>6300</v>
+      </c>
+      <c r="O15" s="4">
+        <v>45971</v>
+      </c>
+      <c r="R15" s="3"/>
+      <c r="T15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <f>SUM(T$2:T15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>165</v>
+      </c>
+      <c r="C16" s="2">
+        <v>3.125E-2</v>
       </c>
       <c r="E16">
         <f t="shared" si="0"/>
@@ -2386,16 +2938,48 @@
       </c>
       <c r="F16">
         <f>SUM(E$2:E16)</f>
-        <v>19500</v>
+        <v>25110</v>
       </c>
       <c r="H16">
         <f>F16-SUM(G$2:G16)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>5610</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L16">
+        <v>45</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="2"/>
+        <v>1350</v>
+      </c>
+      <c r="N16">
+        <f>SUM(M$2:M16)</f>
+        <v>7650</v>
+      </c>
+      <c r="O16" s="4">
+        <v>45971</v>
+      </c>
+      <c r="R16" s="3"/>
+      <c r="T16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <f>SUM(T$2:T16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A17">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" s="2">
+        <v>5.2083333333333336E-2</v>
       </c>
       <c r="E17">
         <f t="shared" si="0"/>
@@ -2403,436 +2987,1668 @@
       </c>
       <c r="F17">
         <f>SUM(E$2:E17)</f>
-        <v>19500</v>
+        <v>25110</v>
       </c>
       <c r="H17">
         <f>F17-SUM(G$2:G17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+        <v>5610</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L17">
+        <v>75</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="2"/>
+        <v>2250</v>
+      </c>
+      <c r="N17">
+        <f>SUM(M$2:M17)</f>
+        <v>9900</v>
+      </c>
+      <c r="O17" s="1">
+        <v>45953</v>
+      </c>
+      <c r="R17" s="3"/>
+      <c r="T17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <f>SUM(T$2:T17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A18">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C18" s="2">
+        <v>5.9722222222222225E-2</v>
       </c>
       <c r="E18">
-        <f t="shared" ref="E18:E42" si="1">D18*30</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F18">
         <f>SUM(E$2:E18)</f>
-        <v>19500</v>
+        <v>25110</v>
       </c>
       <c r="H18">
         <f>F18-SUM(G$2:G18)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+        <v>5610</v>
+      </c>
+      <c r="K18" s="3"/>
+      <c r="M18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <f>SUM(M$2:M18)</f>
+        <v>9900</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="S18">
+        <v>86</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="1"/>
+        <v>3010</v>
+      </c>
+      <c r="U18">
+        <f>SUM(T$2:T18)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A19">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>146</v>
+      </c>
+      <c r="C19" s="2">
+        <v>4.4444444444444446E-2</v>
+      </c>
+      <c r="D19">
+        <v>64</v>
       </c>
       <c r="E19">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1920</v>
       </c>
       <c r="F19">
         <f>SUM(E$2:E19)</f>
-        <v>19500</v>
+        <v>27030</v>
       </c>
       <c r="H19">
         <f>F19-SUM(G$2:G19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+        <v>7530</v>
+      </c>
+      <c r="I19" t="s">
+        <v>161</v>
+      </c>
+      <c r="K19" s="3"/>
+      <c r="M19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <f>SUM(M$2:M19)</f>
+        <v>9900</v>
+      </c>
+      <c r="R19" s="3"/>
+      <c r="T19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <f>SUM(T$2:T19)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A20">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>147</v>
+      </c>
+      <c r="C20" s="2">
+        <v>4.0972222222222222E-2</v>
+      </c>
+      <c r="D20">
+        <v>59</v>
       </c>
       <c r="E20">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1770</v>
       </c>
       <c r="F20">
         <f>SUM(E$2:E20)</f>
-        <v>19500</v>
+        <v>28800</v>
       </c>
       <c r="H20">
         <f>F20-SUM(G$2:G20)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+        <v>9300</v>
+      </c>
+      <c r="I20" t="s">
+        <v>161</v>
+      </c>
+      <c r="K20" s="3"/>
+      <c r="M20">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <f>SUM(M$2:M20)</f>
+        <v>9900</v>
+      </c>
+      <c r="R20" s="3"/>
+      <c r="T20">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <f>SUM(T$2:T20)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A21">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21" s="2">
+        <v>4.3055555555555555E-2</v>
+      </c>
+      <c r="D21">
+        <v>62</v>
       </c>
       <c r="E21">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1860</v>
       </c>
       <c r="F21">
         <f>SUM(E$2:E21)</f>
-        <v>19500</v>
+        <v>30660</v>
       </c>
       <c r="H21">
         <f>F21-SUM(G$2:G21)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+        <v>11160</v>
+      </c>
+      <c r="I21" t="s">
+        <v>161</v>
+      </c>
+      <c r="K21" s="3"/>
+      <c r="M21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <f>SUM(M$2:M21)</f>
+        <v>9900</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <f>SUM(T$2:T21)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A22">
-        <v>20</v>
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C22" s="2">
+        <v>4.583333333333333E-2</v>
+      </c>
+      <c r="D22">
+        <v>66</v>
       </c>
       <c r="E22">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1980</v>
       </c>
       <c r="F22">
         <f>SUM(E$2:E22)</f>
-        <v>19500</v>
+        <v>32640</v>
       </c>
       <c r="H22">
         <f>F22-SUM(G$2:G22)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13140</v>
+      </c>
+      <c r="I22" t="s">
+        <v>161</v>
+      </c>
+      <c r="K22" s="3"/>
+      <c r="M22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N22">
+        <f>SUM(M$2:M22)</f>
+        <v>9900</v>
+      </c>
+      <c r="T22">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U22">
+        <f>SUM(T$2:T22)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A23">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>150</v>
+      </c>
+      <c r="C23" s="2">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="D23">
+        <v>48</v>
       </c>
       <c r="E23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1440</v>
       </c>
       <c r="F23">
         <f>SUM(E$2:E23)</f>
-        <v>19500</v>
+        <v>34080</v>
       </c>
       <c r="H23">
         <f>F23-SUM(G$2:G23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+        <v>14580</v>
+      </c>
+      <c r="I23" t="s">
+        <v>161</v>
+      </c>
+      <c r="K23" s="3"/>
+      <c r="M23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <f>SUM(M$2:M23)</f>
+        <v>9900</v>
+      </c>
+      <c r="T23">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <f>SUM(T$2:T23)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A24">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>151</v>
+      </c>
+      <c r="C24" s="2">
+        <v>4.3749999999999997E-2</v>
+      </c>
+      <c r="D24">
+        <v>63</v>
       </c>
       <c r="E24">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1890</v>
       </c>
       <c r="F24">
         <f>SUM(E$2:E24)</f>
-        <v>19500</v>
+        <v>35970</v>
+      </c>
+      <c r="G24">
+        <v>12660</v>
       </c>
       <c r="H24">
         <f>F24-SUM(G$2:G24)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3810</v>
+      </c>
+      <c r="I24" t="s">
+        <v>161</v>
+      </c>
+      <c r="J24">
+        <v>3</v>
+      </c>
+      <c r="K24" s="3"/>
+      <c r="M24">
+        <f>L24*30</f>
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <f>SUM(M$2:M24)</f>
+        <v>9900</v>
+      </c>
+      <c r="T24">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <f>SUM(T$2:T24)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A25">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" s="2">
+        <v>4.6527777777777779E-2</v>
+      </c>
+      <c r="D25">
+        <v>67</v>
       </c>
       <c r="E25">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>2010</v>
       </c>
       <c r="F25">
         <f>SUM(E$2:E25)</f>
-        <v>19500</v>
+        <v>37980</v>
       </c>
       <c r="H25">
         <f>F25-SUM(G$2:G25)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+        <v>5820</v>
+      </c>
+      <c r="I25" t="s">
+        <v>161</v>
+      </c>
+      <c r="J25">
+        <v>3</v>
+      </c>
+      <c r="M25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <f>SUM(M$2:M25)</f>
+        <v>9900</v>
+      </c>
+      <c r="T25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U25">
+        <f>SUM(T$2:T25)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C26" s="2">
+        <v>4.3749999999999997E-2</v>
+      </c>
+      <c r="D26">
+        <v>63</v>
       </c>
       <c r="E26">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1890</v>
       </c>
       <c r="F26">
         <f>SUM(E$2:E26)</f>
-        <v>19500</v>
+        <v>39870</v>
       </c>
       <c r="H26">
         <f>F26-SUM(G$2:G26)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+        <v>7710</v>
+      </c>
+      <c r="I26" t="s">
+        <v>161</v>
+      </c>
+      <c r="J26">
+        <v>3</v>
+      </c>
+      <c r="M26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N26">
+        <f>SUM(M$2:M26)</f>
+        <v>9900</v>
+      </c>
+      <c r="T26">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U26">
+        <f>SUM(T$2:T26)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A27">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27" s="2">
+        <v>3.9583333333333331E-2</v>
+      </c>
+      <c r="D27">
+        <v>57</v>
       </c>
       <c r="E27">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1710</v>
       </c>
       <c r="F27">
         <f>SUM(E$2:E27)</f>
-        <v>19500</v>
+        <v>41580</v>
       </c>
       <c r="H27">
         <f>F27-SUM(G$2:G27)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+        <v>9420</v>
+      </c>
+      <c r="I27" t="s">
+        <v>161</v>
+      </c>
+      <c r="J27">
+        <v>3</v>
+      </c>
+      <c r="M27">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N27">
+        <f>SUM(M$2:M27)</f>
+        <v>9900</v>
+      </c>
+      <c r="T27">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U27">
+        <f>SUM(T$2:T27)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>26</v>
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>155</v>
+      </c>
+      <c r="C28" s="2">
+        <v>4.027777777777778E-2</v>
+      </c>
+      <c r="D28">
+        <v>58</v>
       </c>
       <c r="E28">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1740</v>
       </c>
       <c r="F28">
         <f>SUM(E$2:E28)</f>
-        <v>19500</v>
+        <v>43320</v>
       </c>
       <c r="H28">
         <f>F28-SUM(G$2:G28)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+        <v>11160</v>
+      </c>
+      <c r="I28" t="s">
+        <v>161</v>
+      </c>
+      <c r="J28">
+        <v>3</v>
+      </c>
+      <c r="M28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N28">
+        <f>SUM(M$2:M28)</f>
+        <v>9900</v>
+      </c>
+      <c r="T28">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U28">
+        <f>SUM(T$2:T28)</f>
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A29">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="B29" t="s">
+        <v>156</v>
+      </c>
+      <c r="C29" s="2">
+        <v>3.6805555555555557E-2</v>
       </c>
       <c r="E29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F29">
         <f>SUM(E$2:E29)</f>
-        <v>19500</v>
+        <v>43320</v>
       </c>
       <c r="H29">
         <f>F29-SUM(G$2:G29)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+        <v>11160</v>
+      </c>
+      <c r="M29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <f>SUM(M$2:M29)</f>
+        <v>9900</v>
+      </c>
+      <c r="R29" t="s">
+        <v>177</v>
+      </c>
+      <c r="S29">
+        <v>53</v>
+      </c>
+      <c r="T29">
+        <f t="shared" si="1"/>
+        <v>1855</v>
+      </c>
+      <c r="U29">
+        <f>SUM(T$2:T29)</f>
+        <v>4865</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A30">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>157</v>
+      </c>
+      <c r="C30" s="2">
+        <v>2.2222222222222223E-2</v>
+      </c>
+      <c r="D30">
+        <v>32</v>
       </c>
       <c r="E30">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>960</v>
       </c>
       <c r="F30">
         <f>SUM(E$2:E30)</f>
-        <v>19500</v>
+        <v>44280</v>
       </c>
       <c r="H30">
         <f>F30-SUM(G$2:G30)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+        <v>12120</v>
+      </c>
+      <c r="I30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="M30">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N30">
+        <f>SUM(M$2:M30)</f>
+        <v>9900</v>
+      </c>
+      <c r="T30">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U30">
+        <f>SUM(T$2:T30)</f>
+        <v>4865</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A31">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
+        <v>158</v>
+      </c>
+      <c r="C31" s="2">
+        <v>5.0694444444444445E-2</v>
       </c>
       <c r="E31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F31">
         <f>SUM(E$2:E31)</f>
-        <v>19500</v>
+        <v>44280</v>
       </c>
       <c r="H31">
         <f>F31-SUM(G$2:G31)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+        <v>12120</v>
+      </c>
+      <c r="M31">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N31">
+        <f>SUM(M$2:M31)</f>
+        <v>9900</v>
+      </c>
+      <c r="R31" t="s">
+        <v>177</v>
+      </c>
+      <c r="S31">
+        <v>73</v>
+      </c>
+      <c r="T31">
+        <f t="shared" si="1"/>
+        <v>2555</v>
+      </c>
+      <c r="U31">
+        <f>SUM(T$2:T31)</f>
+        <v>7420</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A32">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>159</v>
+      </c>
+      <c r="C32" s="2">
+        <v>4.027777777777778E-2</v>
+      </c>
+      <c r="D32">
+        <v>58</v>
       </c>
       <c r="E32">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1740</v>
       </c>
       <c r="F32">
         <f>SUM(E$2:E32)</f>
-        <v>19500</v>
+        <v>46020</v>
       </c>
       <c r="H32">
         <f>F32-SUM(G$2:G32)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13860</v>
+      </c>
+      <c r="I32" t="s">
+        <v>161</v>
+      </c>
+      <c r="J32">
+        <v>3</v>
+      </c>
+      <c r="M32">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N32">
+        <f>SUM(M$2:M32)</f>
+        <v>9900</v>
+      </c>
+      <c r="T32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U32">
+        <f>SUM(T$2:T32)</f>
+        <v>7420</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A33">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" s="2">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="D33">
+        <v>55</v>
       </c>
       <c r="E33">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1650</v>
       </c>
       <c r="F33">
         <f>SUM(E$2:E33)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H33">
         <f>F33-SUM(G$2:G33)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+        <v>15510</v>
+      </c>
+      <c r="I33" t="s">
+        <v>161</v>
+      </c>
+      <c r="J33">
+        <v>3</v>
+      </c>
+      <c r="M33">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N33">
+        <f>SUM(M$2:M33)</f>
+        <v>9900</v>
+      </c>
+      <c r="T33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U33">
+        <f>SUM(T$2:T33)</f>
+        <v>7420</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A34">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>169</v>
+      </c>
+      <c r="C34" s="2">
+        <v>4.7222222222222221E-2</v>
       </c>
       <c r="E34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F34">
         <f>SUM(E$2:E34)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H34">
         <f>F34-SUM(G$2:G34)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+        <v>15510</v>
+      </c>
+      <c r="M34">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N34">
+        <f>SUM(M$2:M34)</f>
+        <v>9900</v>
+      </c>
+      <c r="R34" t="s">
+        <v>177</v>
+      </c>
+      <c r="S34">
+        <v>55</v>
+      </c>
+      <c r="T34">
+        <f t="shared" si="1"/>
+        <v>1925</v>
+      </c>
+      <c r="U34">
+        <f>SUM(T$2:T34)</f>
+        <v>9345</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A35">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="B35" t="s">
+        <v>170</v>
+      </c>
+      <c r="C35" s="2">
+        <v>4.5138888888888888E-2</v>
       </c>
       <c r="E35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F35">
         <f>SUM(E$2:E35)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H35">
         <f>F35-SUM(G$2:G35)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+        <v>15510</v>
+      </c>
+      <c r="R35" t="s">
+        <v>177</v>
+      </c>
+      <c r="S35">
+        <v>65</v>
+      </c>
+      <c r="T35">
+        <f t="shared" si="1"/>
+        <v>2275</v>
+      </c>
+      <c r="U35">
+        <f>SUM(T$2:T35)</f>
+        <v>11620</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>34</v>
+        <v>33</v>
+      </c>
+      <c r="B36" t="s">
+        <v>171</v>
+      </c>
+      <c r="C36" s="2">
+        <v>5.1388888888888887E-2</v>
       </c>
       <c r="E36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F36">
         <f>SUM(E$2:E36)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H36">
         <f>F36-SUM(G$2:G36)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+        <v>15510</v>
+      </c>
+      <c r="R36" t="s">
+        <v>177</v>
+      </c>
+      <c r="S36">
+        <v>74</v>
+      </c>
+      <c r="T36">
+        <f t="shared" si="1"/>
+        <v>2590</v>
+      </c>
+      <c r="U36">
+        <f>SUM(T$2:T36)</f>
+        <v>14210</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A37">
-        <v>35</v>
+        <v>34</v>
+      </c>
+      <c r="B37" t="s">
+        <v>172</v>
+      </c>
+      <c r="C37" s="2">
+        <v>3.5416666666666666E-2</v>
       </c>
       <c r="E37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F37">
         <f>SUM(E$2:E37)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H37">
         <f>F37-SUM(G$2:G37)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+        <v>15510</v>
+      </c>
+      <c r="R37" t="s">
+        <v>177</v>
+      </c>
+      <c r="S37">
+        <v>51</v>
+      </c>
+      <c r="T37">
+        <f t="shared" si="1"/>
+        <v>1785</v>
+      </c>
+      <c r="U37">
+        <f>SUM(T$2:T37)</f>
+        <v>15995</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A38">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="B38" t="s">
+        <v>166</v>
+      </c>
+      <c r="C38" s="2">
+        <v>4.027777777777778E-2</v>
       </c>
       <c r="E38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F38">
         <f>SUM(E$2:E38)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H38">
         <f>F38-SUM(G$2:G38)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+        <v>15510</v>
+      </c>
+      <c r="R38" t="s">
+        <v>177</v>
+      </c>
+      <c r="S38">
+        <v>58</v>
+      </c>
+      <c r="T38">
+        <f t="shared" si="1"/>
+        <v>2030</v>
+      </c>
+      <c r="U38">
+        <f>SUM(T$2:T38)</f>
+        <v>18025</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A39">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B39" t="s">
+        <v>167</v>
+      </c>
+      <c r="C39" s="2">
+        <v>3.8194444444444448E-2</v>
       </c>
       <c r="E39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F39">
         <f>SUM(E$2:E39)</f>
-        <v>19500</v>
+        <v>47670</v>
       </c>
       <c r="H39">
         <f>F39-SUM(G$2:G39)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A40">
-        <v>38</v>
-      </c>
-      <c r="E40">
+        <v>15510</v>
+      </c>
+      <c r="R39" t="s">
+        <v>177</v>
+      </c>
+      <c r="S39">
+        <v>55</v>
+      </c>
+      <c r="T39">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F40">
-        <f>SUM(E$2:E40)</f>
-        <v>19500</v>
-      </c>
-      <c r="H40">
-        <f>F40-SUM(G$2:G40)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41">
-        <v>39</v>
-      </c>
-      <c r="E41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F41">
-        <f>SUM(E$2:E41)</f>
-        <v>19500</v>
-      </c>
-      <c r="H41">
-        <f>F41-SUM(G$2:G41)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A42">
-        <v>40</v>
-      </c>
-      <c r="E42">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F42">
-        <f>SUM(E$2:E42)</f>
-        <v>19500</v>
-      </c>
-      <c r="H42">
-        <f>F42-SUM(G$2:G42)</f>
-        <v>0</v>
+        <v>1925</v>
+      </c>
+      <c r="U39">
+        <f>SUM(T$2:T39)</f>
+        <v>19950</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2732A19D-5FC2-4197-88B3-ABDEAAAB6EBD}">
+  <dimension ref="A1:E37"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" t="s">
+        <v>197</v>
+      </c>
+      <c r="D3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C7" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C10" t="s">
+        <v>197</v>
+      </c>
+      <c r="D10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>198</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>185</v>
+      </c>
+      <c r="C12" t="s">
+        <v>197</v>
+      </c>
+      <c r="D12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>197</v>
+      </c>
+      <c r="D14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>198</v>
+      </c>
+      <c r="D15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" t="s">
+        <v>197</v>
+      </c>
+      <c r="D16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>197</v>
+      </c>
+      <c r="D17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" t="s">
+        <v>197</v>
+      </c>
+      <c r="D18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" t="s">
+        <v>197</v>
+      </c>
+      <c r="D19" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>181</v>
+      </c>
+      <c r="C20" t="s">
+        <v>197</v>
+      </c>
+      <c r="D20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>187</v>
+      </c>
+      <c r="C21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D21" t="s">
+        <v>59</v>
+      </c>
+      <c r="E21" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>181</v>
+      </c>
+      <c r="C22" t="s">
+        <v>198</v>
+      </c>
+      <c r="D22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>188</v>
+      </c>
+      <c r="C23" t="s">
+        <v>197</v>
+      </c>
+      <c r="D23" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>189</v>
+      </c>
+      <c r="C24" t="s">
+        <v>198</v>
+      </c>
+      <c r="D24" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>190</v>
+      </c>
+      <c r="C25" t="s">
+        <v>198</v>
+      </c>
+      <c r="D25" t="s">
+        <v>59</v>
+      </c>
+      <c r="E25" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" t="s">
+        <v>197</v>
+      </c>
+      <c r="D26" t="s">
+        <v>103</v>
+      </c>
+      <c r="E26" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>191</v>
+      </c>
+      <c r="C27" t="s">
+        <v>197</v>
+      </c>
+      <c r="D27" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>192</v>
+      </c>
+      <c r="C28" t="s">
+        <v>198</v>
+      </c>
+      <c r="D28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E28" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>193</v>
+      </c>
+      <c r="C29" t="s">
+        <v>197</v>
+      </c>
+      <c r="D29" t="s">
+        <v>58</v>
+      </c>
+      <c r="E29" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C30" t="s">
+        <v>198</v>
+      </c>
+      <c r="D30" t="s">
+        <v>59</v>
+      </c>
+      <c r="E30" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
+        <v>198</v>
+      </c>
+      <c r="D31" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>116</v>
+      </c>
+      <c r="C32" t="s">
+        <v>197</v>
+      </c>
+      <c r="D32" t="s">
+        <v>58</v>
+      </c>
+      <c r="E32" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" t="s">
+        <v>198</v>
+      </c>
+      <c r="D33" t="s">
+        <v>62</v>
+      </c>
+      <c r="E33" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>194</v>
+      </c>
+      <c r="C34" t="s">
+        <v>197</v>
+      </c>
+      <c r="D34" t="s">
+        <v>62</v>
+      </c>
+      <c r="E34" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>195</v>
+      </c>
+      <c r="C35" t="s">
+        <v>198</v>
+      </c>
+      <c r="D35" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>196</v>
+      </c>
+      <c r="C36" t="s">
+        <v>197</v>
+      </c>
+      <c r="D36" t="s">
+        <v>62</v>
+      </c>
+      <c r="E36" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>195</v>
+      </c>
+      <c r="C37" t="s">
+        <v>197</v>
+      </c>
+      <c r="D37" t="s">
+        <v>62</v>
+      </c>
+      <c r="E37" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>